<commit_message>
Convert to static site
</commit_message>
<xml_diff>
--- a/static/data/Extended-Indexes.xlsx
+++ b/static/data/Extended-Indexes.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ444"/>
+  <dimension ref="A1:AQ445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -51616,6 +51616,139 @@
         <v>4.5</v>
       </c>
     </row>
+    <row r="445">
+      <c r="A445" s="1" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B445" t="n">
+        <v>0</v>
+      </c>
+      <c r="C445" t="n">
+        <v>7.692307692307693</v>
+      </c>
+      <c r="D445" t="n">
+        <v>44.82758620689656</v>
+      </c>
+      <c r="E445" t="n">
+        <v>76.92307692307693</v>
+      </c>
+      <c r="F445" t="n">
+        <v>14.28571428571428</v>
+      </c>
+      <c r="G445" t="n">
+        <v>45870.83333333334</v>
+      </c>
+      <c r="H445" t="n">
+        <v>0.9523809523809524</v>
+      </c>
+      <c r="I445" t="n">
+        <v>-0.1052631578947369</v>
+      </c>
+      <c r="J445" t="n">
+        <v>0.7954545454545454</v>
+      </c>
+      <c r="K445" t="n">
+        <v>1.052631578947368</v>
+      </c>
+      <c r="L445" t="n">
+        <v>1.825</v>
+      </c>
+      <c r="M445" t="n">
+        <v>2.175</v>
+      </c>
+      <c r="N445" t="n">
+        <v>3.708333333333333</v>
+      </c>
+      <c r="O445" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="P445" t="n">
+        <v>72.88</v>
+      </c>
+      <c r="Q445" t="n">
+        <v>34.78947368421053</v>
+      </c>
+      <c r="R445" t="n">
+        <v>-0.04375000000000009</v>
+      </c>
+      <c r="S445" t="n">
+        <v>-0.8647058823529412</v>
+      </c>
+      <c r="T445" t="n">
+        <v>0.8058823529411767</v>
+      </c>
+      <c r="U445" t="n">
+        <v>1.352941176470588</v>
+      </c>
+      <c r="V445" t="n">
+        <v>45.99999999999999</v>
+      </c>
+      <c r="W445" t="n">
+        <v>58.62068965517241</v>
+      </c>
+      <c r="X445" t="n">
+        <v>54.16666666666666</v>
+      </c>
+      <c r="Y445" t="n">
+        <v>39.28571428571428</v>
+      </c>
+      <c r="Z445" t="n">
+        <v>28</v>
+      </c>
+      <c r="AA445" t="n">
+        <v>68.96551724137932</v>
+      </c>
+      <c r="AB445" t="n">
+        <v>76</v>
+      </c>
+      <c r="AC445" t="n">
+        <v>68.96551724137932</v>
+      </c>
+      <c r="AD445" t="n">
+        <v>41.66666666666667</v>
+      </c>
+      <c r="AE445" t="n">
+        <v>22.125</v>
+      </c>
+      <c r="AF445" t="n">
+        <v>30.04</v>
+      </c>
+      <c r="AG445" t="n">
+        <v>48.27586206896552</v>
+      </c>
+      <c r="AH445" t="n">
+        <v>52</v>
+      </c>
+      <c r="AI445" t="n">
+        <v>75.86206896551724</v>
+      </c>
+      <c r="AJ445" t="n">
+        <v>75</v>
+      </c>
+      <c r="AK445" t="n">
+        <v>58.62068965517241</v>
+      </c>
+      <c r="AL445" t="n">
+        <v>32</v>
+      </c>
+      <c r="AM445" t="n">
+        <v>6.583333333333334</v>
+      </c>
+      <c r="AN445" t="n">
+        <v>8.925925925925926</v>
+      </c>
+      <c r="AO445" t="n">
+        <v>6.65263157894737</v>
+      </c>
+      <c r="AP445" t="n">
+        <v>7.175925925925927</v>
+      </c>
+      <c r="AQ445" t="n">
+        <v>5.828947368421054</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
August 2026 data update
</commit_message>
<xml_diff>
--- a/static/data/Extended-Indexes.xlsx
+++ b/static/data/Extended-Indexes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ447"/>
+  <dimension ref="A1:AQ448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52001,6 +52001,139 @@
         <v>2.202142857142857</v>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B448" t="n">
+        <v>0</v>
+      </c>
+      <c r="C448" t="n">
+        <v>0</v>
+      </c>
+      <c r="D448" t="n">
+        <v>30</v>
+      </c>
+      <c r="E448" t="n">
+        <v>55.55555555555556</v>
+      </c>
+      <c r="F448" t="n">
+        <v>0</v>
+      </c>
+      <c r="G448" t="n">
+        <v>51833.33333333334</v>
+      </c>
+      <c r="H448" t="n">
+        <v>-0.6666666666666667</v>
+      </c>
+      <c r="I448" t="n">
+        <v>1.0625</v>
+      </c>
+      <c r="J448" t="n">
+        <v>3</v>
+      </c>
+      <c r="K448" t="n">
+        <v>0.4375000000000001</v>
+      </c>
+      <c r="L448" t="n">
+        <v>3.571428571428571</v>
+      </c>
+      <c r="M448" t="n">
+        <v>-1.6875</v>
+      </c>
+      <c r="N448" t="n">
+        <v>3.714285714285714</v>
+      </c>
+      <c r="O448" t="n">
+        <v>1.444444444444445</v>
+      </c>
+      <c r="P448" t="n">
+        <v>71.125</v>
+      </c>
+      <c r="Q448" t="n">
+        <v>32.31250000000001</v>
+      </c>
+      <c r="R448" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="S448" t="n">
+        <v>5.666666666666667</v>
+      </c>
+      <c r="T448" t="n">
+        <v>4</v>
+      </c>
+      <c r="U448" t="n">
+        <v>4</v>
+      </c>
+      <c r="V448" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="W448" t="n">
+        <v>50</v>
+      </c>
+      <c r="X448" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="Y448" t="n">
+        <v>20</v>
+      </c>
+      <c r="Z448" t="n">
+        <v>27.77777777777778</v>
+      </c>
+      <c r="AA448" t="n">
+        <v>70</v>
+      </c>
+      <c r="AB448" t="n">
+        <v>61.11111111111111</v>
+      </c>
+      <c r="AC448" t="n">
+        <v>60</v>
+      </c>
+      <c r="AD448" t="n">
+        <v>38.88888888888889</v>
+      </c>
+      <c r="AE448" t="n">
+        <v>20.6</v>
+      </c>
+      <c r="AF448" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="AG448" t="n">
+        <v>80</v>
+      </c>
+      <c r="AH448" t="n">
+        <v>77.77777777777779</v>
+      </c>
+      <c r="AI448" t="n">
+        <v>90</v>
+      </c>
+      <c r="AJ448" t="n">
+        <v>66.66666666666666</v>
+      </c>
+      <c r="AK448" t="n">
+        <v>77.77777777777779</v>
+      </c>
+      <c r="AL448" t="n">
+        <v>33.33333333333333</v>
+      </c>
+      <c r="AM448" t="n">
+        <v>3.509999999999999</v>
+      </c>
+      <c r="AN448" t="n">
+        <v>4.357142857142858</v>
+      </c>
+      <c r="AO448" t="n">
+        <v>1.0625</v>
+      </c>
+      <c r="AP448" t="n">
+        <v>4.5625</v>
+      </c>
+      <c r="AQ448" t="n">
+        <v>2.875</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>